<commit_message>
Made Questionare sections into pages
</commit_message>
<xml_diff>
--- a/questionnaire/household_survey.xlsx
+++ b/questionnaire/household_survey.xlsx
@@ -556,7 +556,11 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -835,7 +839,11 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1243,7 +1251,11 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -2585,7 +2597,11 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
@@ -2982,7 +2998,11 @@
           <t>${room_type} != 'outside_security'</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
@@ -3184,7 +3204,11 @@
           <t>${room_type} != 'outside_security' and ${room_weekend_same} = 'no'</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
@@ -3466,7 +3490,11 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
@@ -4026,7 +4054,11 @@
           <t>${always_on} = 'no' and ${weekday_frequency} != 'never'</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
@@ -4357,7 +4389,11 @@
           <t>${always_on} = 'no' and ${weekend_frequency} != 'never' and (${weekday_frequency} = 'never' or ${weekend_same_as_weekday} = 'no')</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
@@ -4679,7 +4715,11 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
@@ -5316,7 +5356,11 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
@@ -5622,7 +5666,11 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
@@ -9392,7 +9440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9416,6 +9464,11 @@
           <t>default_language</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>style</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9430,12 +9483,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026100301</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>English</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>pages</t>
         </is>
       </c>
     </row>

</xml_diff>